<commit_message>
docs: finalize Sprint 2 test documentation and deviations
</commit_message>
<xml_diff>
--- a/docs/Team10_TestCases_RTM.xlsx
+++ b/docs/Team10_TestCases_RTM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shrey\Downloads\vehicle_parking_system\vehicle_parking_system\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7BAA379-EBAF-4BE2-8EEF-67B4F5BDE085}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FDD2E72-2E2C-4F3D-BAF7-812E40816653}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="11370" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="816" uniqueCount="370">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="828" uniqueCount="374">
   <si>
     <t>Test Execution Summary</t>
   </si>
@@ -1146,7 +1146,19 @@
     <t>Checkout only for owner/admin</t>
   </si>
   <si>
-    <t>- Automated results: the team's pytest run on main reported 97 passed, 0 failed (supplied by the team). Update the Result column on the 'Automated Tests' sheet after each run.</t>
+    <t>- Automated results: the team's pytest run on main reported 99 passed, 0 failed (supplied by the team). Update the Result column on the 'Automated Tests' sheet after each run.</t>
+  </si>
+  <si>
+    <t>test_csrf.py</t>
+  </si>
+  <si>
+    <t>test_post_without_csrf_token_is_rejected</t>
+  </si>
+  <si>
+    <t>TC-Sec-04: POST request without a CSRF token is rejected</t>
+  </si>
+  <si>
+    <t>TC-Sec-04: POST request with a valid CSRF token is accepted</t>
   </si>
 </sst>
 </file>
@@ -1221,7 +1233,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -1244,11 +1256,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF999999"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF999999"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1265,6 +1288,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1603,7 +1632,7 @@
         <v>7</v>
       </c>
       <c r="B10" s="3">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.35">
@@ -1611,7 +1640,7 @@
         <v>2</v>
       </c>
       <c r="B11" s="3">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.35">
@@ -2629,7 +2658,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:H78"/>
+  <dimension ref="A1:H80"/>
   <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -4600,6 +4629,58 @@
       </c>
       <c r="H78" s="7" t="s">
         <v>212</v>
+      </c>
+    </row>
+    <row r="79" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A79" s="10">
+        <v>75</v>
+      </c>
+      <c r="B79" s="10" t="s">
+        <v>370</v>
+      </c>
+      <c r="C79" s="10" t="s">
+        <v>371</v>
+      </c>
+      <c r="D79" s="10" t="s">
+        <v>197</v>
+      </c>
+      <c r="E79" s="10">
+        <v>1</v>
+      </c>
+      <c r="F79" s="10" t="s">
+        <v>171</v>
+      </c>
+      <c r="G79" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="H79" s="10" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="80" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A80" s="10">
+        <v>76</v>
+      </c>
+      <c r="B80" s="10" t="s">
+        <v>370</v>
+      </c>
+      <c r="C80" s="10" t="s">
+        <v>371</v>
+      </c>
+      <c r="D80" s="10" t="s">
+        <v>197</v>
+      </c>
+      <c r="E80" s="10">
+        <v>1</v>
+      </c>
+      <c r="F80" s="10" t="s">
+        <v>171</v>
+      </c>
+      <c r="G80" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="H80" s="10" t="s">
+        <v>373</v>
       </c>
     </row>
   </sheetData>

</xml_diff>